<commit_message>
feat: add example Excel templates and configurations and update app logic
</commit_message>
<xml_diff>
--- a/example/e1_config.xlsx
+++ b/example/e1_config.xlsx
@@ -422,7 +422,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>template_e1.xlsx</t>
+          <t>../../template_e1.xlsx</t>
         </is>
       </c>
     </row>
@@ -481,15 +481,11 @@
           <t>2010_qwerty</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2010</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>20101</t>
-        </is>
+      <c r="B5" t="n">
+        <v>201005</v>
+      </c>
+      <c r="C5" t="n">
+        <v>20101</v>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
@@ -518,15 +514,11 @@
           <t>2020_qwerty</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>20201</t>
-        </is>
+      <c r="B6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C6" t="n">
+        <v>20201</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: implement dedicated load and save utilities for Excel configuration templates
</commit_message>
<xml_diff>
--- a/example/e1_config.xlsx
+++ b/example/e1_config.xlsx
@@ -422,7 +422,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>../../template_e1.xlsx</t>
+          <t>../../../template_e1.xlsx</t>
         </is>
       </c>
     </row>
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="F5" t="n">
         <v>2</v>

</xml_diff>